<commit_message>
Update products and modal cards
</commit_message>
<xml_diff>
--- a/storage/products.xlsx
+++ b/storage/products.xlsx
@@ -2795,7 +2795,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -2804,7 +2804,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="6" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="6" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="6"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -5583,7 +5582,7 @@
       <c r="N36" t="s">
         <v>33</v>
       </c>
-      <c r="O36" s="5" t="s">
+      <c r="O36" s="4" t="s">
         <v>147</v>
       </c>
       <c r="P36" t="s">
@@ -5651,7 +5650,7 @@
       <c r="N37" t="s">
         <v>33</v>
       </c>
-      <c r="O37" s="5" t="s">
+      <c r="O37" s="4" t="s">
         <v>147</v>
       </c>
       <c r="P37" t="s">
@@ -5787,7 +5786,7 @@
       <c r="N39" t="s">
         <v>33</v>
       </c>
-      <c r="O39" s="5" t="s">
+      <c r="O39" s="4" t="s">
         <v>158</v>
       </c>
       <c r="P39" t="s">
@@ -5855,7 +5854,7 @@
       <c r="N40" t="s">
         <v>33</v>
       </c>
-      <c r="O40" s="6" t="s">
+      <c r="O40" s="5" t="s">
         <v>163</v>
       </c>
       <c r="P40" t="s">
@@ -5923,7 +5922,7 @@
       <c r="N41" t="s">
         <v>33</v>
       </c>
-      <c r="O41" s="6" t="s">
+      <c r="O41" s="5" t="s">
         <v>168</v>
       </c>
       <c r="P41" t="s">
@@ -5962,7 +5961,7 @@
         <v>24</v>
       </c>
       <c r="E42" t="s">
-        <v>66</v>
+        <v>143</v>
       </c>
       <c r="F42" t="s">
         <v>165</v>
@@ -5991,7 +5990,7 @@
       <c r="N42" t="s">
         <v>33</v>
       </c>
-      <c r="O42" s="6" t="s">
+      <c r="O42" s="5" t="s">
         <v>172</v>
       </c>
       <c r="P42" t="s">
@@ -6059,7 +6058,6 @@
       <c r="N43" t="s">
         <v>33</v>
       </c>
-      <c r="O43"/>
       <c r="P43" t="s">
         <v>29</v>
       </c>

</xml_diff>